<commit_message>
fix: update some script
</commit_message>
<xml_diff>
--- a/data/proteomics/ProMassRatio_across_compartment_NCB.xlsx
+++ b/data/proteomics/ProMassRatio_across_compartment_NCB.xlsx
@@ -2455,70 +2455,70 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>0.02160407921970471</v>
+        <v>0.01757863244382366</v>
       </c>
       <c r="D27" t="n">
-        <v>0.01461152020419359</v>
+        <v>0.01177881259218376</v>
       </c>
       <c r="E27" t="n">
-        <v>0.02103145720796474</v>
+        <v>0.01688457480179846</v>
       </c>
       <c r="F27" t="n">
-        <v>0.02125404107969346</v>
+        <v>0.01606615520001587</v>
       </c>
       <c r="G27" t="n">
-        <v>0.02246750724871094</v>
+        <v>0.01653203714326237</v>
       </c>
       <c r="H27" t="n">
-        <v>0.01597591495080488</v>
+        <v>0.0134494450837891</v>
       </c>
       <c r="I27" t="n">
-        <v>0.01951563297739833</v>
+        <v>0.01495329132117749</v>
       </c>
       <c r="J27" t="n">
-        <v>0.01982672522565734</v>
+        <v>0.01516410011789097</v>
       </c>
       <c r="K27" t="n">
-        <v>0.02175306752395888</v>
+        <v>0.01681270194749483</v>
       </c>
       <c r="L27" t="n">
-        <v>0.0191730170980907</v>
+        <v>0.01509394609934514</v>
       </c>
       <c r="M27" t="n">
-        <v>0.02033380577450473</v>
+        <v>0.0155264071086134</v>
       </c>
       <c r="N27" t="n">
-        <v>0.0226438908789496</v>
+        <v>0.01712396077849517</v>
       </c>
       <c r="O27" t="n">
-        <v>0.02234172080302028</v>
+        <v>0.016674239514736</v>
       </c>
       <c r="P27" t="n">
-        <v>0.02979969394460556</v>
+        <v>0.02416297264424862</v>
       </c>
       <c r="Q27" t="n">
-        <v>0.030696403556217</v>
+        <v>0.02328638242529111</v>
       </c>
       <c r="R27" t="n">
-        <v>0.02885273973795942</v>
+        <v>0.0216473125196204</v>
       </c>
       <c r="S27" t="n">
-        <v>0.02502976360986367</v>
+        <v>0.01924298677102506</v>
       </c>
       <c r="T27" t="n">
-        <v>0.02711491775191053</v>
+        <v>0.02064373399060444</v>
       </c>
       <c r="U27" t="n">
-        <v>0.02817344082815094</v>
+        <v>0.02111308698399664</v>
       </c>
       <c r="V27" t="n">
-        <v>0.02874156010322902</v>
+        <v>0.02215719669362924</v>
       </c>
       <c r="W27" t="n">
-        <v>0.02672060374705813</v>
+        <v>0.02020461058052933</v>
       </c>
       <c r="X27" t="n">
-        <v>0.02700441259003436</v>
+        <v>0.02103146281215684</v>
       </c>
     </row>
     <row r="28">

</xml_diff>